<commit_message>
Add machine learning model to predict next 5 years eps growth
</commit_message>
<xml_diff>
--- a/data/AMZN/AMZN.xlsx
+++ b/data/AMZN/AMZN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wayne\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{213C5575-B09E-4366-B99F-CF970F079131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51D4F5D4-BEAC-4413-A02B-0BB57A729845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{977960B1-1FAF-4A15-A498-13B5BEAFE3E6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{977960B1-1FAF-4A15-A498-13B5BEAFE3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="9">
   <si>
     <t>ticker</t>
   </si>
@@ -53,16 +53,10 @@
     <t>net_income</t>
   </si>
   <si>
-    <t>ebitda</t>
-  </si>
-  <si>
     <t>eps</t>
   </si>
   <si>
     <t>basic_average_shares</t>
-  </si>
-  <si>
-    <t>research_and_development</t>
   </si>
   <si>
     <t>total_expenses</t>
@@ -440,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D8FB664-2497-46B3-A203-B65314FB20BE}">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
@@ -448,13 +442,13 @@
     <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -479,622 +473,576 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2">
-        <v>2001</v>
+        <v>2003</v>
       </c>
       <c r="C2">
-        <v>3122</v>
+        <v>5264</v>
+      </c>
+      <c r="D2">
+        <v>270</v>
       </c>
       <c r="E2">
-        <v>-567</v>
+        <v>35</v>
+      </c>
+      <c r="F2">
+        <v>0.09</v>
       </c>
       <c r="G2">
-        <v>-1.56</v>
+        <v>395</v>
       </c>
       <c r="H2">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>2002</v>
+        <v>2004</v>
       </c>
       <c r="C3">
-        <v>3933</v>
+        <v>6921</v>
+      </c>
+      <c r="D3">
+        <v>440</v>
       </c>
       <c r="E3">
-        <v>-149</v>
+        <v>588</v>
+      </c>
+      <c r="F3">
+        <v>1.45</v>
       </c>
       <c r="G3">
-        <v>-0.39</v>
+        <v>406</v>
       </c>
       <c r="H3">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4">
-        <v>2003</v>
+        <v>2005</v>
       </c>
       <c r="C4">
-        <v>5264</v>
+        <v>8490</v>
       </c>
       <c r="D4">
-        <v>270</v>
+        <v>432</v>
       </c>
       <c r="E4">
-        <v>35</v>
+        <v>359</v>
+      </c>
+      <c r="F4">
+        <v>0.87</v>
       </c>
       <c r="G4">
-        <v>0.09</v>
+        <v>412</v>
       </c>
       <c r="H4">
-        <v>395</v>
-      </c>
-      <c r="J4">
-        <v>987</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5">
-        <v>2004</v>
+        <v>2006</v>
       </c>
       <c r="C5">
-        <v>6921</v>
+        <v>10711</v>
       </c>
       <c r="D5">
-        <v>440</v>
+        <v>389</v>
       </c>
       <c r="E5">
-        <v>588</v>
+        <v>190</v>
+      </c>
+      <c r="F5">
+        <v>0.46</v>
       </c>
       <c r="G5">
-        <v>1.45</v>
+        <v>416</v>
       </c>
       <c r="H5">
-        <v>406</v>
-      </c>
-      <c r="J5">
-        <v>1162</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <v>2067</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6">
-        <v>2005</v>
+        <v>2007</v>
       </c>
       <c r="C6">
-        <v>8490</v>
+        <v>14835</v>
       </c>
       <c r="D6">
-        <v>432</v>
+        <v>655</v>
       </c>
       <c r="E6">
-        <v>359</v>
+        <v>476</v>
+      </c>
+      <c r="F6">
+        <v>1.1499999999999999</v>
       </c>
       <c r="G6">
-        <v>0.87</v>
+        <v>413</v>
       </c>
       <c r="H6">
-        <v>412</v>
-      </c>
-      <c r="J6">
-        <v>1607</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <v>2698</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>2006</v>
+        <v>2008</v>
       </c>
       <c r="C7">
-        <v>10711</v>
+        <v>19166</v>
       </c>
       <c r="D7">
-        <v>389</v>
+        <v>842</v>
       </c>
       <c r="E7">
-        <v>190</v>
+        <v>645</v>
+      </c>
+      <c r="F7">
+        <v>1.52</v>
       </c>
       <c r="G7">
-        <v>0.46</v>
+        <v>423</v>
       </c>
       <c r="H7">
-        <v>416</v>
-      </c>
-      <c r="J7">
-        <v>2067</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>3428</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8">
-        <v>2007</v>
+        <v>2009</v>
       </c>
       <c r="C8">
-        <v>14835</v>
+        <v>24509</v>
       </c>
       <c r="D8">
-        <v>655</v>
+        <v>1129</v>
       </c>
       <c r="E8">
-        <v>476</v>
+        <v>902</v>
+      </c>
+      <c r="F8">
+        <v>2.08</v>
       </c>
       <c r="G8">
-        <v>1.1499999999999999</v>
+        <v>433</v>
       </c>
       <c r="H8">
-        <v>413</v>
-      </c>
-      <c r="J8">
-        <v>2698</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <v>23380</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9">
-        <v>2008</v>
+        <v>2010</v>
       </c>
       <c r="C9">
-        <v>19166</v>
+        <v>34204</v>
       </c>
       <c r="D9">
-        <v>842</v>
+        <v>1406</v>
       </c>
       <c r="E9">
-        <v>645</v>
+        <v>1152</v>
+      </c>
+      <c r="F9">
+        <v>2.58</v>
       </c>
       <c r="G9">
-        <v>1.52</v>
+        <v>447</v>
       </c>
       <c r="H9">
-        <v>423</v>
-      </c>
-      <c r="J9">
-        <v>3428</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+        <v>32378</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B10">
-        <v>2009</v>
+        <v>2011</v>
       </c>
       <c r="C10">
-        <v>24509</v>
+        <v>48077</v>
       </c>
       <c r="D10">
-        <v>1129</v>
+        <v>862</v>
       </c>
       <c r="E10">
-        <v>902</v>
+        <v>631</v>
+      </c>
+      <c r="F10">
+        <v>1.39</v>
       </c>
       <c r="G10">
-        <v>2.08</v>
+        <v>453</v>
       </c>
       <c r="H10">
-        <v>433</v>
-      </c>
-      <c r="J10">
-        <v>23380</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47215</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11">
-        <v>2010</v>
+        <v>2012</v>
       </c>
       <c r="C11">
-        <v>34204</v>
+        <v>61093</v>
       </c>
       <c r="D11">
-        <v>1406</v>
+        <v>676</v>
       </c>
       <c r="E11">
-        <v>1152</v>
+        <v>-39</v>
+      </c>
+      <c r="F11">
+        <v>-0.09</v>
       </c>
       <c r="G11">
-        <v>2.58</v>
+        <v>453</v>
       </c>
       <c r="H11">
-        <v>447</v>
-      </c>
-      <c r="J11">
-        <v>32378</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>60417</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
-        <v>2011</v>
+        <v>2013</v>
       </c>
       <c r="C12">
-        <v>48077</v>
+        <v>74452</v>
       </c>
       <c r="D12">
-        <v>862</v>
+        <v>745</v>
       </c>
       <c r="E12">
-        <v>631</v>
+        <v>274</v>
+      </c>
+      <c r="F12">
+        <v>0.6</v>
       </c>
       <c r="G12">
-        <v>1.39</v>
+        <v>457</v>
       </c>
       <c r="H12">
-        <v>453</v>
-      </c>
-      <c r="J12">
-        <v>47215</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>73707</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B13">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="C13">
-        <v>61093</v>
+        <v>88988</v>
       </c>
       <c r="D13">
-        <v>676</v>
+        <v>178</v>
       </c>
       <c r="E13">
-        <v>-39</v>
+        <v>-241</v>
+      </c>
+      <c r="F13">
+        <v>-0.52</v>
       </c>
       <c r="G13">
-        <v>-0.09</v>
+        <v>462</v>
       </c>
       <c r="H13">
-        <v>453</v>
-      </c>
-      <c r="J13">
-        <v>60417</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>88810</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B14">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="C14">
-        <v>74452</v>
+        <v>107006</v>
       </c>
       <c r="D14">
-        <v>745</v>
+        <v>2233</v>
       </c>
       <c r="E14">
-        <v>274</v>
+        <v>596</v>
+      </c>
+      <c r="F14">
+        <v>1.28</v>
       </c>
       <c r="G14">
-        <v>0.6</v>
+        <v>467</v>
       </c>
       <c r="H14">
-        <v>457</v>
-      </c>
-      <c r="J14">
-        <v>73707</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <v>104773</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B15">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="C15">
-        <v>88988</v>
+        <v>135987</v>
       </c>
       <c r="D15">
-        <v>178</v>
+        <v>4186</v>
       </c>
       <c r="E15">
-        <v>-241</v>
+        <v>2371</v>
+      </c>
+      <c r="F15">
+        <v>5.01</v>
       </c>
       <c r="G15">
-        <v>-0.52</v>
+        <v>474</v>
       </c>
       <c r="H15">
-        <v>462</v>
-      </c>
-      <c r="J15">
-        <v>88810</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>131801</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B16">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="C16">
-        <v>107006</v>
+        <v>177866</v>
       </c>
       <c r="D16">
-        <v>2233</v>
+        <v>4106</v>
       </c>
       <c r="E16">
-        <v>596</v>
+        <v>3033</v>
+      </c>
+      <c r="F16">
+        <v>6.32</v>
       </c>
       <c r="G16">
-        <v>1.28</v>
+        <v>480</v>
       </c>
       <c r="H16">
-        <v>467</v>
-      </c>
-      <c r="J16">
-        <v>104773</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>173760</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B17">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="C17">
-        <v>135987</v>
+        <v>232887</v>
       </c>
       <c r="D17">
-        <v>4186</v>
+        <v>12421</v>
       </c>
       <c r="E17">
-        <v>2371</v>
+        <v>10073</v>
+      </c>
+      <c r="F17">
+        <v>20.68</v>
       </c>
       <c r="G17">
-        <v>5.01</v>
+        <v>487</v>
       </c>
       <c r="H17">
-        <v>474</v>
-      </c>
-      <c r="J17">
-        <v>131801</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+        <v>220466</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B18">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="C18">
-        <v>177866</v>
+        <v>280522</v>
       </c>
       <c r="D18">
-        <v>4106</v>
+        <v>14541</v>
       </c>
       <c r="E18">
-        <v>3033</v>
+        <v>11588</v>
+      </c>
+      <c r="F18">
+        <v>23.46</v>
       </c>
       <c r="G18">
-        <v>6.32</v>
+        <v>494</v>
       </c>
       <c r="H18">
-        <v>480</v>
-      </c>
-      <c r="J18">
-        <v>173760</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+        <v>265981</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B19">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="C19">
-        <v>232887</v>
+        <v>386064</v>
       </c>
       <c r="D19">
-        <v>12421</v>
+        <v>22899</v>
       </c>
       <c r="E19">
-        <v>10073</v>
+        <v>21331</v>
+      </c>
+      <c r="F19">
+        <v>42.64</v>
       </c>
       <c r="G19">
-        <v>20.68</v>
+        <v>500</v>
       </c>
       <c r="H19">
-        <v>487</v>
-      </c>
-      <c r="J19">
-        <v>220466</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+        <v>363165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B20">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C20">
-        <v>280522</v>
+        <v>469822</v>
       </c>
       <c r="D20">
-        <v>14541</v>
+        <v>24879</v>
       </c>
       <c r="E20">
-        <v>11588</v>
+        <v>33364</v>
+      </c>
+      <c r="F20">
+        <v>65.959999999999994</v>
       </c>
       <c r="G20">
-        <v>23.46</v>
+        <v>506</v>
       </c>
       <c r="H20">
-        <v>494</v>
-      </c>
-      <c r="J20">
-        <v>265981</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+        <v>444943</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B21">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C21">
-        <v>386064</v>
+        <v>513983</v>
       </c>
       <c r="D21">
-        <v>22899</v>
+        <v>12248</v>
       </c>
       <c r="E21">
-        <v>21331</v>
+        <v>-2722</v>
+      </c>
+      <c r="F21">
+        <v>-0.27</v>
       </c>
       <c r="G21">
-        <v>42.64</v>
+        <v>10189</v>
       </c>
       <c r="H21">
-        <v>500</v>
-      </c>
-      <c r="J21">
-        <v>363165</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+        <v>501735</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B22">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C22">
-        <v>469822</v>
+        <v>574785</v>
       </c>
       <c r="D22">
-        <v>24879</v>
+        <v>36852</v>
       </c>
       <c r="E22">
-        <v>33364</v>
+        <v>30425</v>
+      </c>
+      <c r="F22">
+        <v>2.95</v>
       </c>
       <c r="G22">
-        <v>65.959999999999994</v>
+        <v>10304</v>
       </c>
       <c r="H22">
-        <v>506</v>
-      </c>
-      <c r="J22">
-        <v>444943</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+        <v>537933</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B23">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C23">
-        <v>513983</v>
+        <v>637959</v>
       </c>
       <c r="D23">
-        <v>12248</v>
+        <v>68593</v>
       </c>
       <c r="E23">
-        <v>-2722</v>
+        <v>59248</v>
+      </c>
+      <c r="F23">
+        <v>5.66</v>
       </c>
       <c r="G23">
-        <v>-0.27</v>
+        <v>10473</v>
       </c>
       <c r="H23">
-        <v>10189</v>
-      </c>
-      <c r="J23">
-        <v>501735</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24">
-        <v>2023</v>
-      </c>
-      <c r="C24">
-        <v>574785</v>
-      </c>
-      <c r="D24">
-        <v>36852</v>
-      </c>
-      <c r="E24">
-        <v>30425</v>
-      </c>
-      <c r="G24">
-        <v>2.95</v>
-      </c>
-      <c r="H24">
-        <v>10304</v>
-      </c>
-      <c r="J24">
-        <v>537933</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25">
-        <v>2024</v>
-      </c>
-      <c r="C25">
-        <v>637959</v>
-      </c>
-      <c r="D25">
-        <v>68593</v>
-      </c>
-      <c r="E25">
-        <v>59248</v>
-      </c>
-      <c r="G25">
-        <v>5.66</v>
-      </c>
-      <c r="H25">
-        <v>10473</v>
-      </c>
-      <c r="J25">
         <v>569366</v>
       </c>
     </row>

</xml_diff>